<commit_message>
Ajoute l'onglet Ma wish list
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NX4jhiWVddeZCTEunnUA3A
</commit_message>
<xml_diff>
--- a/idees_cadeaux.xlsx
+++ b/idees_cadeaux.xlsx
@@ -10,12 +10,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Côté Maman" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Côté Papa" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Copine &amp; sa famille" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Récap budget" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ma wish list" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Récap budget" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Côté Maman'!$A$3:$G$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Côté Papa'!$A$3:$G$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Copine &amp; sa famille'!$A$3:$G$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Ma wish list'!$A$3:$G$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -51,7 +53,7 @@
       <sz val="16"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -83,6 +85,11 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E69138"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -110,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -134,8 +141,11 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1557,6 +1567,515 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>⭐ Ma wish list</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Catégorie</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Priorité</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>Prix (€)</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>Lien</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>Offert par</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>Reçu ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Glacière transport repas midi</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Divers</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="n"/>
+      <c r="D4" s="12" t="n"/>
+      <c r="E4" s="11" t="n"/>
+      <c r="F4" s="11" t="n"/>
+      <c r="G4" s="11" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Compressport R2V2</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Course / Trail</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="n"/>
+      <c r="D5" s="12" t="n"/>
+      <c r="E5" s="11" t="n"/>
+      <c r="F5" s="11" t="n"/>
+      <c r="G5" s="11" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Gel Meltonic</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Course / Trail</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="12" t="n"/>
+      <c r="E6" s="11" t="n"/>
+      <c r="F6" s="11" t="n"/>
+      <c r="G6" s="11" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Débardeur course</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Course / Trail</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="12" t="n"/>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="11" t="n"/>
+      <c r="G7" s="11" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Écouteurs</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="12" t="n"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n"/>
+      <c r="G8" s="11" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Garmin HRM Pro Plus</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="12" t="n"/>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="11" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Chaussettes trail</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Course / Trail</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="12" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
+      <c r="G10" s="11" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Vêtements course à pied</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Course / Trail</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="12" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+      <c r="G11" s="11" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Casquette</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Course / Trail</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Bâtons de trail</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Course / Trail</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="12" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="11" t="n"/>
+      <c r="G13" s="11" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Sac de sport grand under</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="12" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+      <c r="G14" s="11" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>PS5 + Madden</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="12" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
+      <c r="G15" s="11" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Maillot NFL</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="12" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Oreiller ergonomique</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Maison</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="12" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>Raquette padel</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="12" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Montre</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="12" t="n"/>
+      <c r="E19" s="11" t="n"/>
+      <c r="F19" s="11" t="n"/>
+      <c r="G19" s="11" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Box U2</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Divers</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="12" t="n"/>
+      <c r="E20" s="11" t="n"/>
+      <c r="F20" s="11" t="n"/>
+      <c r="G20" s="11" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>Chaussures On</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Course / Trail</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="n"/>
+      <c r="D21" s="12" t="n"/>
+      <c r="E21" s="11" t="n"/>
+      <c r="F21" s="11" t="n"/>
+      <c r="G21" s="11" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Coque téléphone</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="n"/>
+      <c r="D22" s="12" t="n"/>
+      <c r="E22" s="11" t="n"/>
+      <c r="F22" s="11" t="n"/>
+      <c r="G22" s="11" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="n"/>
+      <c r="B23" s="11" t="n"/>
+      <c r="C23" s="11" t="n"/>
+      <c r="D23" s="12" t="n"/>
+      <c r="E23" s="11" t="n"/>
+      <c r="F23" s="11" t="n"/>
+      <c r="G23" s="11" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="n"/>
+      <c r="B24" s="11" t="n"/>
+      <c r="C24" s="11" t="n"/>
+      <c r="D24" s="12" t="n"/>
+      <c r="E24" s="11" t="n"/>
+      <c r="F24" s="11" t="n"/>
+      <c r="G24" s="11" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="n"/>
+      <c r="B25" s="11" t="n"/>
+      <c r="C25" s="11" t="n"/>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="11" t="n"/>
+      <c r="F25" s="11" t="n"/>
+      <c r="G25" s="11" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="n"/>
+      <c r="B26" s="11" t="n"/>
+      <c r="C26" s="11" t="n"/>
+      <c r="D26" s="12" t="n"/>
+      <c r="E26" s="11" t="n"/>
+      <c r="F26" s="11" t="n"/>
+      <c r="G26" s="11" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="n"/>
+      <c r="B27" s="11" t="n"/>
+      <c r="C27" s="11" t="n"/>
+      <c r="D27" s="12" t="n"/>
+      <c r="E27" s="11" t="n"/>
+      <c r="F27" s="11" t="n"/>
+      <c r="G27" s="11" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="n"/>
+      <c r="B28" s="11" t="n"/>
+      <c r="C28" s="11" t="n"/>
+      <c r="D28" s="12" t="n"/>
+      <c r="E28" s="11" t="n"/>
+      <c r="F28" s="11" t="n"/>
+      <c r="G28" s="11" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="n"/>
+      <c r="B29" s="11" t="n"/>
+      <c r="C29" s="11" t="n"/>
+      <c r="D29" s="12" t="n"/>
+      <c r="E29" s="11" t="n"/>
+      <c r="F29" s="11" t="n"/>
+      <c r="G29" s="11" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="n"/>
+      <c r="B30" s="11" t="n"/>
+      <c r="C30" s="11" t="n"/>
+      <c r="D30" s="12" t="n"/>
+      <c r="E30" s="11" t="n"/>
+      <c r="F30" s="11" t="n"/>
+      <c r="G30" s="11" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="n"/>
+      <c r="B31" s="11" t="n"/>
+      <c r="C31" s="11" t="n"/>
+      <c r="D31" s="12" t="n"/>
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="11" t="n"/>
+      <c r="G31" s="11" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="n"/>
+      <c r="B32" s="11" t="n"/>
+      <c r="C32" s="11" t="n"/>
+      <c r="D32" s="12" t="n"/>
+      <c r="E32" s="11" t="n"/>
+      <c r="F32" s="11" t="n"/>
+      <c r="G32" s="11" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="n"/>
+      <c r="B33" s="11" t="n"/>
+      <c r="C33" s="11" t="n"/>
+      <c r="D33" s="12" t="n"/>
+      <c r="E33" s="11" t="n"/>
+      <c r="F33" s="11" t="n"/>
+      <c r="G33" s="11" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:G33"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A4:G33">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$G4="Oui"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="3">
+    <dataValidation sqref="C4:C33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Haute,Moyenne,Basse"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F4:F33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Maman,Papa,Frère,Copine,Famille copine,Autre"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G4:G33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Oui,Non"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1568,7 +2087,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>💰 Récap budget</t>
         </is>
@@ -1607,11 +2126,11 @@
           <t>Côté Maman</t>
         </is>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="14">
         <f>SUM('Côté Maman'!D4:D28)</f>
         <v/>
       </c>
-      <c r="C4" s="11">
+      <c r="C4" s="14">
         <f>SUM('Côté Maman'!E4:E28)</f>
         <v/>
       </c>
@@ -1630,11 +2149,11 @@
           <t>Côté Papa</t>
         </is>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="14">
         <f>SUM('Côté Papa'!D4:D28)</f>
         <v/>
       </c>
-      <c r="C5" s="11">
+      <c r="C5" s="14">
         <f>SUM('Côté Papa'!E4:E28)</f>
         <v/>
       </c>
@@ -1653,11 +2172,11 @@
           <t>Copine &amp; sa famille</t>
         </is>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="14">
         <f>SUM('Copine &amp; sa famille'!D4:D28)</f>
         <v/>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="14">
         <f>SUM('Copine &amp; sa famille'!E4:E28)</f>
         <v/>
       </c>
@@ -1671,7 +2190,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -1684,11 +2203,11 @@
         <f>SUM(C4:C6)</f>
         <v/>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="15">
         <f>SUM(D4:D6)</f>
         <v/>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="15">
         <f>SUM(E4:E6)</f>
         <v/>
       </c>
@@ -1699,7 +2218,7 @@
           <t>Budget max (à saisir) :</t>
         </is>
       </c>
-      <c r="B9" s="13" t="n"/>
+      <c r="B9" s="16" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1707,7 +2226,7 @@
           <t>Reste :</t>
         </is>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="14">
         <f>IF(B9="","",B9-C7)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Ajoute les liens montres et nouvelles idées dans la wish list
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NX4jhiWVddeZCTEunnUA3A
</commit_message>
<xml_diff>
--- a/idees_cadeaux.xlsx
+++ b/idees_cadeaux.xlsx
@@ -2442,7 +2442,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Glacière transport repas midi</t>
         </is>
@@ -2453,10 +2453,10 @@
         </is>
       </c>
       <c r="C4" s="10" t="n"/>
-      <c r="D4" s="10" t="n"/>
+      <c r="D4" s="6" t="n"/>
       <c r="E4" s="10" t="n"/>
       <c r="F4" s="10" t="n"/>
-      <c r="G4" s="10" t="n"/>
+      <c r="G4" s="6" t="n"/>
       <c r="H4" s="11">
         <f>IF($E4="Papa",COUNTIF($E$4:$E4,"Papa"),"")</f>
         <v/>
@@ -2467,7 +2467,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Compressport R2V2</t>
         </is>
@@ -2478,10 +2478,10 @@
         </is>
       </c>
       <c r="C5" s="10" t="n"/>
-      <c r="D5" s="10" t="n"/>
+      <c r="D5" s="6" t="n"/>
       <c r="E5" s="10" t="n"/>
       <c r="F5" s="10" t="n"/>
-      <c r="G5" s="10" t="n"/>
+      <c r="G5" s="6" t="n"/>
       <c r="H5" s="11">
         <f>IF($E5="Papa",COUNTIF($E$4:$E5,"Papa"),"")</f>
         <v/>
@@ -2492,7 +2492,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Gel Meltonic</t>
         </is>
@@ -2503,10 +2503,10 @@
         </is>
       </c>
       <c r="C6" s="10" t="n"/>
-      <c r="D6" s="10" t="n"/>
+      <c r="D6" s="6" t="n"/>
       <c r="E6" s="10" t="n"/>
       <c r="F6" s="10" t="n"/>
-      <c r="G6" s="10" t="n"/>
+      <c r="G6" s="6" t="n"/>
       <c r="H6" s="11">
         <f>IF($E6="Papa",COUNTIF($E$4:$E6,"Papa"),"")</f>
         <v/>
@@ -2517,7 +2517,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Débardeur course</t>
         </is>
@@ -2528,10 +2528,10 @@
         </is>
       </c>
       <c r="C7" s="10" t="n"/>
-      <c r="D7" s="10" t="n"/>
+      <c r="D7" s="6" t="n"/>
       <c r="E7" s="10" t="n"/>
       <c r="F7" s="10" t="n"/>
-      <c r="G7" s="10" t="n"/>
+      <c r="G7" s="6" t="n"/>
       <c r="H7" s="11">
         <f>IF($E7="Papa",COUNTIF($E$4:$E7,"Papa"),"")</f>
         <v/>
@@ -2542,7 +2542,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Écouteurs</t>
         </is>
@@ -2553,10 +2553,10 @@
         </is>
       </c>
       <c r="C8" s="10" t="n"/>
-      <c r="D8" s="10" t="n"/>
+      <c r="D8" s="6" t="n"/>
       <c r="E8" s="10" t="n"/>
       <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
+      <c r="G8" s="6" t="n"/>
       <c r="H8" s="11">
         <f>IF($E8="Papa",COUNTIF($E$4:$E8,"Papa"),"")</f>
         <v/>
@@ -2567,7 +2567,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Garmin HRM Pro Plus</t>
         </is>
@@ -2578,10 +2578,10 @@
         </is>
       </c>
       <c r="C9" s="10" t="n"/>
-      <c r="D9" s="10" t="n"/>
+      <c r="D9" s="6" t="n"/>
       <c r="E9" s="10" t="n"/>
       <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
+      <c r="G9" s="6" t="n"/>
       <c r="H9" s="11">
         <f>IF($E9="Papa",COUNTIF($E$4:$E9,"Papa"),"")</f>
         <v/>
@@ -2592,7 +2592,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Chaussettes trail</t>
         </is>
@@ -2603,10 +2603,10 @@
         </is>
       </c>
       <c r="C10" s="10" t="n"/>
-      <c r="D10" s="10" t="n"/>
+      <c r="D10" s="6" t="n"/>
       <c r="E10" s="10" t="n"/>
       <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
+      <c r="G10" s="6" t="n"/>
       <c r="H10" s="11">
         <f>IF($E10="Papa",COUNTIF($E$4:$E10,"Papa"),"")</f>
         <v/>
@@ -2617,7 +2617,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Vêtements course à pied</t>
         </is>
@@ -2628,10 +2628,10 @@
         </is>
       </c>
       <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
+      <c r="D11" s="6" t="n"/>
       <c r="E11" s="10" t="n"/>
       <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
+      <c r="G11" s="6" t="n"/>
       <c r="H11" s="11">
         <f>IF($E11="Papa",COUNTIF($E$4:$E11,"Papa"),"")</f>
         <v/>
@@ -2642,7 +2642,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Casquette</t>
         </is>
@@ -2653,10 +2653,10 @@
         </is>
       </c>
       <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
+      <c r="D12" s="6" t="n"/>
       <c r="E12" s="10" t="n"/>
       <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
+      <c r="G12" s="6" t="n"/>
       <c r="H12" s="11">
         <f>IF($E12="Papa",COUNTIF($E$4:$E12,"Papa"),"")</f>
         <v/>
@@ -2667,7 +2667,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Bâtons de trail</t>
         </is>
@@ -2678,10 +2678,10 @@
         </is>
       </c>
       <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
+      <c r="D13" s="6" t="n"/>
       <c r="E13" s="10" t="n"/>
       <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
+      <c r="G13" s="6" t="n"/>
       <c r="H13" s="11">
         <f>IF($E13="Papa",COUNTIF($E$4:$E13,"Papa"),"")</f>
         <v/>
@@ -2692,7 +2692,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Sac de sport grand under</t>
         </is>
@@ -2703,10 +2703,10 @@
         </is>
       </c>
       <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
+      <c r="D14" s="6" t="n"/>
       <c r="E14" s="10" t="n"/>
       <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
+      <c r="G14" s="6" t="n"/>
       <c r="H14" s="11">
         <f>IF($E14="Papa",COUNTIF($E$4:$E14,"Papa"),"")</f>
         <v/>
@@ -2717,7 +2717,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>PS5 + Madden</t>
         </is>
@@ -2728,10 +2728,10 @@
         </is>
       </c>
       <c r="C15" s="10" t="n"/>
-      <c r="D15" s="10" t="n"/>
+      <c r="D15" s="6" t="n"/>
       <c r="E15" s="10" t="n"/>
       <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
+      <c r="G15" s="6" t="n"/>
       <c r="H15" s="11">
         <f>IF($E15="Papa",COUNTIF($E$4:$E15,"Papa"),"")</f>
         <v/>
@@ -2742,7 +2742,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Maillot NFL</t>
         </is>
@@ -2753,10 +2753,10 @@
         </is>
       </c>
       <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
+      <c r="D16" s="6" t="n"/>
       <c r="E16" s="10" t="n"/>
       <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="G16" s="6" t="n"/>
       <c r="H16" s="11">
         <f>IF($E16="Papa",COUNTIF($E$4:$E16,"Papa"),"")</f>
         <v/>
@@ -2767,7 +2767,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Oreiller ergonomique</t>
         </is>
@@ -2778,10 +2778,10 @@
         </is>
       </c>
       <c r="C17" s="10" t="n"/>
-      <c r="D17" s="10" t="n"/>
+      <c r="D17" s="6" t="n"/>
       <c r="E17" s="10" t="n"/>
       <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="n"/>
+      <c r="G17" s="6" t="n"/>
       <c r="H17" s="11">
         <f>IF($E17="Papa",COUNTIF($E$4:$E17,"Papa"),"")</f>
         <v/>
@@ -2792,7 +2792,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Raquette padel</t>
         </is>
@@ -2803,10 +2803,10 @@
         </is>
       </c>
       <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
+      <c r="D18" s="6" t="n"/>
       <c r="E18" s="10" t="n"/>
       <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
+      <c r="G18" s="6" t="n"/>
       <c r="H18" s="11">
         <f>IF($E18="Papa",COUNTIF($E$4:$E18,"Papa"),"")</f>
         <v/>
@@ -2817,9 +2817,9 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>Montre</t>
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Montre (style terrain / rétro)</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
@@ -2828,10 +2828,19 @@
         </is>
       </c>
       <c r="C19" s="10" t="n"/>
-      <c r="D19" s="10" t="n"/>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>https://timex.eu/products/expedition-sierra-40mm-fabric-strap-watch-tw2v22800
+https://charlie-paris.com/products/grx-mecaquartz-chronographe-evo-iii?variant=50144588857670</t>
+        </is>
+      </c>
       <c r="E19" s="10" t="n"/>
       <c r="F19" s="10" t="n"/>
-      <c r="G19" s="10" t="n"/>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Timex Expedition Sierra 40 mm (119 €) / Charlie GRX mecaquartz chrono (395 €)</t>
+        </is>
+      </c>
       <c r="H19" s="11">
         <f>IF($E19="Papa",COUNTIF($E$4:$E19,"Papa"),"")</f>
         <v/>
@@ -2842,7 +2851,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Box U2</t>
         </is>
@@ -2853,10 +2862,10 @@
         </is>
       </c>
       <c r="C20" s="10" t="n"/>
-      <c r="D20" s="10" t="n"/>
+      <c r="D20" s="6" t="n"/>
       <c r="E20" s="10" t="n"/>
       <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
+      <c r="G20" s="6" t="n"/>
       <c r="H20" s="11">
         <f>IF($E20="Papa",COUNTIF($E$4:$E20,"Papa"),"")</f>
         <v/>
@@ -2867,7 +2876,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Chaussures On</t>
         </is>
@@ -2878,10 +2887,10 @@
         </is>
       </c>
       <c r="C21" s="10" t="n"/>
-      <c r="D21" s="10" t="n"/>
+      <c r="D21" s="6" t="n"/>
       <c r="E21" s="10" t="n"/>
       <c r="F21" s="10" t="n"/>
-      <c r="G21" s="10" t="n"/>
+      <c r="G21" s="6" t="n"/>
       <c r="H21" s="11">
         <f>IF($E21="Papa",COUNTIF($E$4:$E21,"Papa"),"")</f>
         <v/>
@@ -2892,7 +2901,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>Coque téléphone</t>
         </is>
@@ -2903,10 +2912,10 @@
         </is>
       </c>
       <c r="C22" s="10" t="n"/>
-      <c r="D22" s="10" t="n"/>
+      <c r="D22" s="6" t="n"/>
       <c r="E22" s="10" t="n"/>
       <c r="F22" s="10" t="n"/>
-      <c r="G22" s="10" t="n"/>
+      <c r="G22" s="6" t="n"/>
       <c r="H22" s="11">
         <f>IF($E22="Papa",COUNTIF($E$4:$E22,"Papa"),"")</f>
         <v/>
@@ -2917,13 +2926,29 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="n"/>
-      <c r="B23" s="10" t="n"/>
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Montre – Timex Expedition North Field Post Solar 41 mm</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
       <c r="C23" s="10" t="n"/>
-      <c r="D23" s="10" t="n"/>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>https://ablogtowatch.com/watch-review-timex-expedition-north-field-post-solar-41mm</t>
+        </is>
+      </c>
       <c r="E23" s="10" t="n"/>
       <c r="F23" s="10" t="n"/>
-      <c r="G23" s="10" t="n"/>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Quartz solaire, 100 m. Lien = test. Env. 170-180 $ (prix à vérifier en €)</t>
+        </is>
+      </c>
       <c r="H23" s="11">
         <f>IF($E23="Papa",COUNTIF($E$4:$E23,"Papa"),"")</f>
         <v/>
@@ -2934,13 +2959,29 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="n"/>
-      <c r="B24" s="10" t="n"/>
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Montre – Citizen Eco-Drive Garrison BM8180</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
       <c r="C24" s="10" t="n"/>
-      <c r="D24" s="10" t="n"/>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>https://longislandwatch.com/products/citizen-eco-drive-garrison-watch-with-black-dial-and-green-strap-bm8180-03e</t>
+        </is>
+      </c>
       <c r="E24" s="10" t="n"/>
       <c r="F24" s="10" t="n"/>
-      <c r="G24" s="10" t="n"/>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Solaire, 37 mm, 100 m. Prix très variable, à vérifier en France</t>
+        </is>
+      </c>
       <c r="H24" s="11">
         <f>IF($E24="Papa",COUNTIF($E$4:$E24,"Papa"),"")</f>
         <v/>
@@ -2951,13 +2992,29 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="n"/>
-      <c r="B25" s="10" t="n"/>
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Montre – Seiko 5 SNK809</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
       <c r="C25" s="10" t="n"/>
-      <c r="D25" s="10" t="n"/>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>https://www.ebay.de/p/24050466267</t>
+        </is>
+      </c>
       <c r="E25" s="10" t="n"/>
       <c r="F25" s="10" t="n"/>
-      <c r="G25" s="10" t="n"/>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Automatique, classique de terrain. Env. 218 € sur une annonce eBay.de, à comparer</t>
+        </is>
+      </c>
       <c r="H25" s="11">
         <f>IF($E25="Papa",COUNTIF($E$4:$E25,"Papa"),"")</f>
         <v/>
@@ -2968,13 +3025,29 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="n"/>
-      <c r="B26" s="10" t="n"/>
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Montre – Hamilton Khaki Field Quartz 40 mm</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
       <c r="C26" s="10" t="n"/>
-      <c r="D26" s="10" t="n"/>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>https://www.thewatchpages.com/watches/hamilton-khaki-field-quartz-40-h68551933</t>
+        </is>
+      </c>
       <c r="E26" s="10" t="n"/>
       <c r="F26" s="10" t="n"/>
-      <c r="G26" s="10" t="n"/>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>Référence du genre, prix catalogue env. 575-595 $ (haut de gamme)</t>
+        </is>
+      </c>
       <c r="H26" s="11">
         <f>IF($E26="Papa",COUNTIF($E$4:$E26,"Papa"),"")</f>
         <v/>
@@ -2985,13 +3058,29 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="n"/>
-      <c r="B27" s="10" t="n"/>
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Montre – Yema Rallygraf (chrono mecaquartz)</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
       <c r="C27" s="10" t="n"/>
-      <c r="D27" s="10" t="n"/>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>https://jamaisvulgaire.com/conseil-montre-homme/meilleure-montre-chronographe-homme-moins-de-500-euros/</t>
+        </is>
+      </c>
       <c r="E27" s="10" t="n"/>
       <c r="F27" s="10" t="n"/>
-      <c r="G27" s="10" t="n"/>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Piste pour un chrono mecaquartz &lt; 500 €. Lien = guide, modèle à vérifier</t>
+        </is>
+      </c>
       <c r="H27" s="11">
         <f>IF($E27="Papa",COUNTIF($E$4:$E27,"Papa"),"")</f>
         <v/>
@@ -3002,13 +3091,13 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="n"/>
+      <c r="A28" s="6" t="n"/>
       <c r="B28" s="10" t="n"/>
       <c r="C28" s="10" t="n"/>
-      <c r="D28" s="10" t="n"/>
+      <c r="D28" s="6" t="n"/>
       <c r="E28" s="10" t="n"/>
       <c r="F28" s="10" t="n"/>
-      <c r="G28" s="10" t="n"/>
+      <c r="G28" s="6" t="n"/>
       <c r="H28" s="11">
         <f>IF($E28="Papa",COUNTIF($E$4:$E28,"Papa"),"")</f>
         <v/>
@@ -3019,13 +3108,13 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="n"/>
+      <c r="A29" s="6" t="n"/>
       <c r="B29" s="10" t="n"/>
       <c r="C29" s="10" t="n"/>
-      <c r="D29" s="10" t="n"/>
+      <c r="D29" s="6" t="n"/>
       <c r="E29" s="10" t="n"/>
       <c r="F29" s="10" t="n"/>
-      <c r="G29" s="10" t="n"/>
+      <c r="G29" s="6" t="n"/>
       <c r="H29" s="11">
         <f>IF($E29="Papa",COUNTIF($E$4:$E29,"Papa"),"")</f>
         <v/>
@@ -3036,13 +3125,13 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="n"/>
+      <c r="A30" s="6" t="n"/>
       <c r="B30" s="10" t="n"/>
       <c r="C30" s="10" t="n"/>
-      <c r="D30" s="10" t="n"/>
+      <c r="D30" s="6" t="n"/>
       <c r="E30" s="10" t="n"/>
       <c r="F30" s="10" t="n"/>
-      <c r="G30" s="10" t="n"/>
+      <c r="G30" s="6" t="n"/>
       <c r="H30" s="11">
         <f>IF($E30="Papa",COUNTIF($E$4:$E30,"Papa"),"")</f>
         <v/>
@@ -3053,13 +3142,13 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="n"/>
+      <c r="A31" s="6" t="n"/>
       <c r="B31" s="10" t="n"/>
       <c r="C31" s="10" t="n"/>
-      <c r="D31" s="10" t="n"/>
+      <c r="D31" s="6" t="n"/>
       <c r="E31" s="10" t="n"/>
       <c r="F31" s="10" t="n"/>
-      <c r="G31" s="10" t="n"/>
+      <c r="G31" s="6" t="n"/>
       <c r="H31" s="11">
         <f>IF($E31="Papa",COUNTIF($E$4:$E31,"Papa"),"")</f>
         <v/>
@@ -3070,13 +3159,13 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="n"/>
+      <c r="A32" s="6" t="n"/>
       <c r="B32" s="10" t="n"/>
       <c r="C32" s="10" t="n"/>
-      <c r="D32" s="10" t="n"/>
+      <c r="D32" s="6" t="n"/>
       <c r="E32" s="10" t="n"/>
       <c r="F32" s="10" t="n"/>
-      <c r="G32" s="10" t="n"/>
+      <c r="G32" s="6" t="n"/>
       <c r="H32" s="11">
         <f>IF($E32="Papa",COUNTIF($E$4:$E32,"Papa"),"")</f>
         <v/>
@@ -3087,13 +3176,13 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="n"/>
+      <c r="A33" s="6" t="n"/>
       <c r="B33" s="10" t="n"/>
       <c r="C33" s="10" t="n"/>
-      <c r="D33" s="10" t="n"/>
+      <c r="D33" s="6" t="n"/>
       <c r="E33" s="10" t="n"/>
       <c r="F33" s="10" t="n"/>
-      <c r="G33" s="10" t="n"/>
+      <c r="G33" s="6" t="n"/>
       <c r="H33" s="11">
         <f>IF($E33="Papa",COUNTIF($E$4:$E33,"Papa"),"")</f>
         <v/>
@@ -3104,13 +3193,13 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="n"/>
+      <c r="A34" s="6" t="n"/>
       <c r="B34" s="10" t="n"/>
       <c r="C34" s="10" t="n"/>
-      <c r="D34" s="10" t="n"/>
+      <c r="D34" s="6" t="n"/>
       <c r="E34" s="10" t="n"/>
       <c r="F34" s="10" t="n"/>
-      <c r="G34" s="10" t="n"/>
+      <c r="G34" s="6" t="n"/>
       <c r="H34" s="11">
         <f>IF($E34="Papa",COUNTIF($E$4:$E34,"Papa"),"")</f>
         <v/>
@@ -3121,13 +3210,13 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="n"/>
+      <c r="A35" s="6" t="n"/>
       <c r="B35" s="10" t="n"/>
       <c r="C35" s="10" t="n"/>
-      <c r="D35" s="10" t="n"/>
+      <c r="D35" s="6" t="n"/>
       <c r="E35" s="10" t="n"/>
       <c r="F35" s="10" t="n"/>
-      <c r="G35" s="10" t="n"/>
+      <c r="G35" s="6" t="n"/>
       <c r="H35" s="11">
         <f>IF($E35="Papa",COUNTIF($E$4:$E35,"Papa"),"")</f>
         <v/>
@@ -3138,13 +3227,13 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="n"/>
+      <c r="A36" s="6" t="n"/>
       <c r="B36" s="10" t="n"/>
       <c r="C36" s="10" t="n"/>
-      <c r="D36" s="10" t="n"/>
+      <c r="D36" s="6" t="n"/>
       <c r="E36" s="10" t="n"/>
       <c r="F36" s="10" t="n"/>
-      <c r="G36" s="10" t="n"/>
+      <c r="G36" s="6" t="n"/>
       <c r="H36" s="11">
         <f>IF($E36="Papa",COUNTIF($E$4:$E36,"Papa"),"")</f>
         <v/>
@@ -3155,13 +3244,13 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="n"/>
+      <c r="A37" s="6" t="n"/>
       <c r="B37" s="10" t="n"/>
       <c r="C37" s="10" t="n"/>
-      <c r="D37" s="10" t="n"/>
+      <c r="D37" s="6" t="n"/>
       <c r="E37" s="10" t="n"/>
       <c r="F37" s="10" t="n"/>
-      <c r="G37" s="10" t="n"/>
+      <c r="G37" s="6" t="n"/>
       <c r="H37" s="11">
         <f>IF($E37="Papa",COUNTIF($E$4:$E37,"Papa"),"")</f>
         <v/>
@@ -3172,13 +3261,13 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="10" t="n"/>
+      <c r="A38" s="6" t="n"/>
       <c r="B38" s="10" t="n"/>
       <c r="C38" s="10" t="n"/>
-      <c r="D38" s="10" t="n"/>
+      <c r="D38" s="6" t="n"/>
       <c r="E38" s="10" t="n"/>
       <c r="F38" s="10" t="n"/>
-      <c r="G38" s="10" t="n"/>
+      <c r="G38" s="6" t="n"/>
       <c r="H38" s="11">
         <f>IF($E38="Papa",COUNTIF($E$4:$E38,"Papa"),"")</f>
         <v/>
@@ -3189,13 +3278,13 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="10" t="n"/>
+      <c r="A39" s="6" t="n"/>
       <c r="B39" s="10" t="n"/>
       <c r="C39" s="10" t="n"/>
-      <c r="D39" s="10" t="n"/>
+      <c r="D39" s="6" t="n"/>
       <c r="E39" s="10" t="n"/>
       <c r="F39" s="10" t="n"/>
-      <c r="G39" s="10" t="n"/>
+      <c r="G39" s="6" t="n"/>
       <c r="H39" s="11">
         <f>IF($E39="Papa",COUNTIF($E$4:$E39,"Papa"),"")</f>
         <v/>
@@ -3206,13 +3295,13 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="10" t="n"/>
+      <c r="A40" s="6" t="n"/>
       <c r="B40" s="10" t="n"/>
       <c r="C40" s="10" t="n"/>
-      <c r="D40" s="10" t="n"/>
+      <c r="D40" s="6" t="n"/>
       <c r="E40" s="10" t="n"/>
       <c r="F40" s="10" t="n"/>
-      <c r="G40" s="10" t="n"/>
+      <c r="G40" s="6" t="n"/>
       <c r="H40" s="11">
         <f>IF($E40="Papa",COUNTIF($E$4:$E40,"Papa"),"")</f>
         <v/>

</xml_diff>

<commit_message>
Ajoute les onglets Si je gagne (début et placements)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NX4jhiWVddeZCTEunnUA3A
</commit_message>
<xml_diff>
--- a/idees_cadeaux.xlsx
+++ b/idees_cadeaux.xlsx
@@ -11,6 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papa" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ma wish list" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Récap" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Si je gagne - Début" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Si je gagne - Placements" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ma wish list'!$A$3:$G$40</definedName>
@@ -21,8 +23,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="7">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0 &quot;€&quot;"/>
+  </numFmts>
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,8 +57,15 @@
       <b val="1"/>
       <sz val="16"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -91,6 +102,16 @@
         <fgColor rgb="00999999"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006AA84F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -118,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -146,6 +167,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3440,4 +3473,836 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>🎰 Si je gagne – les premiers pas (hypothétique)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Informations générales, pas un conseil. Chiffres et règles à revérifier avec un notaire / conseiller indépendant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Étape</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Quand</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Fait ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>1. Ticket</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Signer le ticket, en faire des photos, le ranger en lieu sûr</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Jour J</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>2. Discrétion</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Ne rien dire à personne (ni réseaux sociaux) tant que rien n'est décidé</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Jour J</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>3. Décider le nom</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Voir le tableau « Ticket : à ton nom ou aux deux ? » plus bas, idéalement AVANT de signer</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Jour J</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>4. FDJ</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Contacter la FDJ pour la réclamation et l'accompagnement des gros gagnants</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Jours 1-3</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>5. Équipe</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Choisir un notaire, un conseiller en gestion de patrimoine indépendant (honoraires), un expert-comptable</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Semaine 1</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>6. Banque</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Verser sur un compte, répartir sur plusieurs banques (dépôts garantis à 100 000 € par banque)</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Semaine 1-2</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>7. Pause</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Ne rien dépenser de gros pendant 1 à 3 mois</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Mois 1-3</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>8. Budget plaisir</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Fixer une enveloppe cadeaux / achats plaisir (voir onglet Placements)</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Mois 1</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>9. Famille</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Définir qui reçoit quoi, puis faire des dons encadrés par le notaire</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Mois 1-3</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>10. Protection</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Faire le point sur PACS / mariage, testament, assurance-vie avec bénéficiaire</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Mois 1-3</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>11. Placements</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Investir progressivement selon l'onglet Placements</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Mois 3+</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Ticket : à ton nom ou aux deux ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Option</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Avantages</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Risques / limites</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>À vérifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>À ton nom seul</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Le gain est à toi. Tu gardes la main et tu choisis ensuite à qui donner, de façon encadrée.</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Ta copine n'est pas héritière sans mariage ni testament. Des dons à une personne non mariée ou non pacsée sont taxés lourdement.</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Droits de donation / succession entre non-mariés</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Aux deux noms (copine)</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Le gain est partagé dès le départ.</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Co-propriété : en cas de séparation, c'est compliqué. Aussi une donation indirecte possible. Ça ne règle pas la transmission.</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Notaire AVANT de signer</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>À ton nom + PACS ou mariage</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Le conjoint ou partenaire pacsé est exonéré de droits de succession. Le mariage protège davantage.</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Engagement juridique, régime matrimonial à choisir.</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Contrat de mariage, testament</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>À ton nom + assurance-vie</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Tu désignes qui reçoit, hors succession classique, avec un abattement par bénéficiaire (152 500 € dans le cas général, à vérifier).</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Clause bénéficiaire à rédiger précisément. Fiscalité selon l'âge des versements.</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Clause bénéficiaire avec le notaire</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="D4:D14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Oui,Non"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>💶 Si je gagne – répartition et placements (hypothétique)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Montant gagné (€)</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="n">
+        <v>79000000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Mets les % dans la colonne C. Les montants se calculent seuls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Poste</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Quoi</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>% du gain</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Montant (€)</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Plafond / limite</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Fiscalité (à vérifier)</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Remarques</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Sécurité – comptes</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Plusieurs banques, livrets</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D7" s="17">
+        <f>$B$3*C7</f>
+        <v/>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Garantie 100 000 € par banque. Livret A 22 950 €, LDDS 12 000 €</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Intérêts du Livret A et LDDS exonérés d'impôt</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Réserve de précaution, disponible tout de suite</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Assurance-vie</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Fonds euros + unités de compte</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D8" s="17">
+        <f>$B$3*C8</f>
+        <v/>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Pas de plafond. Plusieurs contrats possibles</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Gains imposés après 8 ans avec abattement 4 600 € (9 200 € couple), puis 7,5 % ou 12,8 % + prélèvements sociaux (~17,2 %, taux à vérifier)</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Bon pour la transmission (abattement par bénéficiaire). Répartir les risques</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>PEA (actions)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Actions européennes, ETF</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D9" s="17">
+        <f>$B$3*C9</f>
+        <v/>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Plafond de versements 150 000 €</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Après 5 ans, plus d'impôt sur les gains (prélèvements sociaux restent)</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Placement long terme, risque de perte</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Compte-titres</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Actions, ETF, obligations</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D10" s="17">
+        <f>$B$3*C10</f>
+        <v/>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Pas de plafond</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Flat tax 30 % (12,8 % + 17,2 %), taux à vérifier</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Souple, mais plus taxé</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Contrat de capitalisation</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Support proche de l'assurance-vie</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D11" s="17">
+        <f>$B$3*C11</f>
+        <v/>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Pas de plafond</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Fiscalité proche de l'assurance-vie</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Utile pour donner / transmettre</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Immobilier</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Résidence principale, locatif</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D12" s="17">
+        <f>$B$3*C12</f>
+        <v/>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>IFI au-delà de 1,3 M € de patrimoine immobilier net</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Revenus fonciers imposés. Résidence principale exonérée de plus-value à la revente</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Demande un notaire, évite l'endettement</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Famille – dons</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Parents, frère, copine et sa famille</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="D13" s="17">
+        <f>$B$3*C13</f>
+        <v/>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Abattement parent-enfant 100 000 € tous les 15 ans. Don d'argent exonéré 31 865 € (donateur &lt; 80 ans, bénéficiaire majeur). Frère/sœur 15 932 €</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Au-delà : droits de donation selon le lien de parenté</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Dons encadrés par le notaire, répartis dans le temps</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Plaisir</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Voyages, montres, PS5, etc.</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D14" s="17">
+        <f>$B$3*C14</f>
+        <v/>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Pas d'impôt sur la dépense</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Fixe-le à l'avance pour ne pas déraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Associations / dons</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Dons à des causes qui comptent</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D15" s="17">
+        <f>$B$3*C15</f>
+        <v/>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Plafond 20 % du revenu imposable</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Réduction d'impôt de 66 % (cas général)</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Optionnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Imprévus / à décider</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Réserve pour décider plus tard</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D16" s="17">
+        <f>$B$3*C16</f>
+        <v/>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Garde une marge</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C17" s="18">
+        <f>SUM(C7:C16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="19">
+        <f>SUM(D7:D16)</f>
+        <v/>
+      </c>
+      <c r="E17">
+        <f>IF(ROUND(C17,4)=1,"✅ 100 %","⚠️ Le total doit faire 100 %")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>Aide pour payer moins d'impôt légalement : enveloppes avantageuses (assurance-vie, PEA, capitalisation), dons échelonnés, bon notaire. Pas d'optimisation agressive.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Refait la répartition Si je gagne selon les objectifs
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NX4jhiWVddeZCTEunnUA3A
</commit_message>
<xml_diff>
--- a/idees_cadeaux.xlsx
+++ b/idees_cadeaux.xlsx
@@ -23,8 +23,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0 &quot;€&quot;"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -139,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -179,6 +180,10 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3860,22 +3865,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
-          <t>💶 Si je gagne – répartition et placements (hypothétique)</t>
+          <t>💶 Si je gagne – ma répartition (hypothétique)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Objectif : vie confortable, aider la famille, voyager, monter des entreprises, beau mariage. Informations générales, à valider avec notaire / conseiller.</t>
         </is>
       </c>
     </row>
@@ -3892,7 +3904,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Mets les % dans la colonne C. Les montants se calculent seuls.</t>
+          <t>Change les % de la colonne C : les montants se calculent seuls.</t>
         </is>
       </c>
     </row>
@@ -3936,16 +3948,16 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Sécurité – comptes</t>
+          <t>Vie confortable</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Plusieurs banques, livrets</t>
-        </is>
-      </c>
-      <c r="C7" s="16" t="n">
-        <v>0.1</v>
+          <t>Maison à deux, voiture, train de vie sans excès</t>
+        </is>
+      </c>
+      <c r="C7" s="21" t="n">
+        <v>0.08</v>
       </c>
       <c r="D7" s="17">
         <f>$B$3*C7</f>
@@ -3953,33 +3965,33 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Garantie 100 000 € par banque. Livret A 22 950 €, LDDS 12 000 €</t>
+          <t>–</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Intérêts du Livret A et LDDS exonérés d'impôt</t>
+          <t>Résidence principale exonérée de plus-value à la revente</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Réserve de précaution, disponible tout de suite</t>
+          <t>Ex. : maison ~2 M€ + budget annuel de ~150 000 € sur 30 ans (~4,5 M€)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Assurance-vie</t>
+          <t>Voyages</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Fonds euros + unités de compte</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="n">
-        <v>0.25</v>
+          <t>Voyages, expériences</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="n">
+        <v>0.03</v>
       </c>
       <c r="D8" s="17">
         <f>$B$3*C8</f>
@@ -3987,33 +3999,33 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Pas de plafond. Plusieurs contrats possibles</t>
+          <t>–</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Gains imposés après 8 ans avec abattement 4 600 € (9 200 € couple), puis 7,5 % ou 12,8 % + prélèvements sociaux (~17,2 %, taux à vérifier)</t>
+          <t>Pas d'impôt sur la dépense</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Bon pour la transmission (abattement par bénéficiaire). Répartir les risques</t>
+          <t>Enveloppe fixée à l'avance</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>PEA (actions)</t>
+          <t>Mariage</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Actions européennes, ETF</t>
-        </is>
-      </c>
-      <c r="C9" s="16" t="n">
-        <v>0.05</v>
+          <t>Un beau mariage</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="n">
+        <v>0.005</v>
       </c>
       <c r="D9" s="17">
         <f>$B$3*C9</f>
@@ -4021,33 +4033,33 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Plafond de versements 150 000 €</t>
+          <t>–</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>Après 5 ans, plus d'impôt sur les gains (prélèvements sociaux restent)</t>
+          <t>–</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Placement long terme, risque de perte</t>
+          <t>~400 000 € de budget large. Avant le mariage : choisir le régime (contrat de mariage)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Compte-titres</t>
+          <t>Famille – dons</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Actions, ETF, obligations</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="n">
-        <v>0.15</v>
+          <t>Parents, frère, sa famille</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="n">
+        <v>0.12</v>
       </c>
       <c r="D10" s="17">
         <f>$B$3*C10</f>
@@ -4055,33 +4067,33 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Pas de plafond</t>
+          <t>Abattement parent-enfant 100 000 € / 15 ans. Don d'argent 31 865 € : enfants, petits-enfants, neveux, PAS les parents</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>Flat tax 30 % (12,8 % + 17,2 %), taux à vérifier</t>
+          <t>Droits de donation au-delà des abattements</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Souple, mais plus taxé</t>
+          <t>Parents traités équitablement. Maison de ta mère en démembrement. Dons échelonnés avec le notaire</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Contrat de capitalisation</t>
+          <t>Entreprises</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Support proche de l'assurance-vie</t>
-        </is>
-      </c>
-      <c r="C11" s="16" t="n">
-        <v>0.1</v>
+          <t>Créer ou racheter des entreprises</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="n">
+        <v>0.08</v>
       </c>
       <c r="D11" s="17">
         <f>$B$3*C11</f>
@@ -4089,33 +4101,33 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Pas de plafond</t>
+          <t>–</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>Fiscalité proche de l'assurance-vie</t>
+          <t>Revenus pro imposés (IR ou IS). Holding possible</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Utile pour donner / transmettre</t>
+          <t>Par tranches, avec un business plan, pas tout d'un coup. Expert-comptable indispensable</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Immobilier</t>
+          <t>Sécurité</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Résidence principale, locatif</t>
-        </is>
-      </c>
-      <c r="C12" s="16" t="n">
-        <v>0.2</v>
+          <t>Fonds euros, comptes à terme, obligations d'État, plusieurs banques</t>
+        </is>
+      </c>
+      <c r="C12" s="21" t="n">
+        <v>0.35</v>
       </c>
       <c r="D12" s="17">
         <f>$B$3*C12</f>
@@ -4123,33 +4135,33 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>IFI au-delà de 1,3 M € de patrimoine immobilier net</t>
+          <t>Dépôts garantis 100 000 € par banque (donc répartir)</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>Revenus fonciers imposés. Résidence principale exonérée de plus-value à la revente</t>
+          <t>Intérêts imposés (flat tax en général)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Demande un notaire, évite l'endettement</t>
+          <t>Le gros du capital reste protégé de la bourse</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Famille – dons</t>
+          <t>Assurance-vie</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Parents, frère, copine et sa famille</t>
-        </is>
-      </c>
-      <c r="C13" s="16" t="n">
-        <v>0.08</v>
+          <t>Contrats multi-assureurs, mixte fonds euros / unités de compte</t>
+        </is>
+      </c>
+      <c r="C13" s="21" t="n">
+        <v>0.1</v>
       </c>
       <c r="D13" s="17">
         <f>$B$3*C13</f>
@@ -4157,33 +4169,33 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Abattement parent-enfant 100 000 € tous les 15 ans. Don d'argent exonéré 31 865 € (donateur &lt; 80 ans, bénéficiaire majeur : enfants, petits-enfants, neveux/nièces, PAS les parents). Frère/sœur 15 932 €</t>
+          <t>Pas de plafond. Répartir entre assureurs (garantie limitée)</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>Au-delà : droits de donation selon le lien de parenté</t>
+          <t>Gains imposés après 8 ans, abattement 4 600 € (9 200 € couple), puis 7,5 % / 12,8 % + prélèvements sociaux (~17,2 %, à vérifier)</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Dons encadrés par le notaire, répartis dans le temps</t>
+          <t>Outil de transmission : bénéficiaires, abattement 152 500 € chacun (versements avant 70 ans, à vérifier)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Plaisir</t>
+          <t>PEA</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Voyages, montres, PS5, etc.</t>
-        </is>
-      </c>
-      <c r="C14" s="16" t="n">
-        <v>0.05</v>
+          <t>Actions européennes, ETF</t>
+        </is>
+      </c>
+      <c r="C14" s="21" t="n">
+        <v>0.002</v>
       </c>
       <c r="D14" s="17">
         <f>$B$3*C14</f>
@@ -4191,33 +4203,33 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Plafond de versements 150 000 €</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>Pas d'impôt sur la dépense</t>
+          <t>Après 5 ans, plus d'impôt sur les gains (prélèvements sociaux restent)</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Fixe-le à l'avance pour ne pas déraper</t>
+          <t>Petit à cette échelle</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Associations / dons</t>
+          <t>Compte-titres</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Dons à des causes qui comptent</t>
-        </is>
-      </c>
-      <c r="C15" s="16" t="n">
-        <v>0.01</v>
+          <t>ETF diversifiés</t>
+        </is>
+      </c>
+      <c r="C15" s="21" t="n">
+        <v>0.078</v>
       </c>
       <c r="D15" s="17">
         <f>$B$3*C15</f>
@@ -4225,33 +4237,33 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Plafond 20 % du revenu imposable</t>
+          <t>Pas de plafond</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Réduction d'impôt de 66 % (cas général)</t>
+          <t>Flat tax 30 % (12,8 % + 17,2 %), à vérifier</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Optionnel</t>
+          <t>Investir progressivement sur 12 à 24 mois</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Imprévus / à décider</t>
+          <t>Immobilier locatif</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Réserve pour décider plus tard</t>
-        </is>
-      </c>
-      <c r="C16" s="16" t="n">
-        <v>0.01</v>
+          <t>Appartements, SCPI</t>
+        </is>
+      </c>
+      <c r="C16" s="21" t="n">
+        <v>0.05</v>
       </c>
       <c r="D16" s="17">
         <f>$B$3*C16</f>
@@ -4259,44 +4271,145 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
+          <t>IFI au-delà de 1,3 M€ de patrimoine immobilier net</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Revenus fonciers imposés</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Passer par un notaire, éviter l'endettement</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Contrat de capitalisation</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Proche de l'assurance-vie</t>
+        </is>
+      </c>
+      <c r="C17" s="21" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D17" s="17">
+        <f>$B$3*C17</f>
+        <v/>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Pas de plafond</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Fiscalité proche de l'assurance-vie</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Utile pour donner ou transmettre</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Associations</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Dons à des causes qui comptent</t>
+        </is>
+      </c>
+      <c r="C18" s="21" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D18" s="17">
+        <f>$B$3*C18</f>
+        <v/>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Plafond 20 % du revenu imposable</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Réduction d'impôt de 66 % (cas général)</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Optionnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Impôts / imprévus</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Marge pour décider plus tard</t>
+        </is>
+      </c>
+      <c r="C19" s="21" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="D19" s="17">
+        <f>$B$3*C19</f>
+        <v/>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
           <t>–</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Garde une marge</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Garde de la marge pour l'impôt sur les revenus des placements</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C17" s="18">
-        <f>SUM(C7:C16)</f>
-        <v/>
-      </c>
-      <c r="D17" s="19">
-        <f>SUM(D7:D16)</f>
-        <v/>
-      </c>
-      <c r="E17">
-        <f>IF(ROUND(C17,4)=1,"✅ 100 %","⚠️ Le total doit faire 100 %")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18"/>
-    <row r="19">
-      <c r="A19" s="20" t="inlineStr">
-        <is>
-          <t>Aide pour payer moins d'impôt légalement : enveloppes avantageuses (assurance-vie, PEA, capitalisation), dons échelonnés, bon notaire. Pas d'optimisation agressive.</t>
+      <c r="C20" s="22">
+        <f>SUM(C7:C19)</f>
+        <v/>
+      </c>
+      <c r="D20" s="19">
+        <f>SUM(D7:D19)</f>
+        <v/>
+      </c>
+      <c r="E20">
+        <f>IF(ROUND(C20,4)=1,"✅ 100 %","⚠️ Le total doit faire 100 %")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="20" t="inlineStr">
+        <is>
+          <t>Pour payer moins d'impôt légalement : enveloppes avantageuses (assurance-vie, PEA, capitalisation), dons échelonnés, bon notaire. Pas d'optimisation agressive.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajoute les étapes mariage et travail dans l'onglet Début
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NX4jhiWVddeZCTEunnUA3A
</commit_message>
<xml_diff>
--- a/idees_cadeaux.xlsx
+++ b/idees_cadeaux.xlsx
@@ -3486,7 +3486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3729,118 +3729,155 @@
       </c>
       <c r="D14" s="6" t="inlineStr"/>
     </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>12. Mariage – contrat</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Décider avec ma copine du régime (séparation de biens, éventuellement avec société d'acquêts pour la maison), contrat chez le notaire AVANT le mariage, + testament / donation entre époux / clause bénéficiaire de l'assurance-vie</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Mois 1-6</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr"/>
+    </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>13. Travail</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Ne pas démissionner tout de suite. Lire ma convention collective (préavis), décider ensuite : démission ou rupture conventionnelle (qui demande l'accord de l'employeur). Rester professionnel, ne pas annoncer le gain</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Mois 3+</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Ticket : à ton nom ou aux deux ?</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Option</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Avantages</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Risques / limites</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>À vérifier</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>À ton nom seul</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>Le gain est à toi. Tu gardes la main et tu choisis ensuite à qui donner, de façon encadrée.</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>Ta copine n'est pas héritière sans mariage ni testament. Des dons à une personne non mariée ou non pacsée sont taxés lourdement.</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>Droits de donation / succession entre non-mariés</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Aux deux noms (copine)</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>Le gain est partagé dès le départ.</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>Co-propriété : en cas de séparation, c'est compliqué. Aussi une donation indirecte possible. Ça ne règle pas la transmission.</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>Notaire AVANT de signer</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>À ton nom + PACS ou mariage</t>
+          <t>À ton nom seul</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Le conjoint ou partenaire pacsé est exonéré de droits de succession. Le mariage protège davantage.</t>
+          <t>Le gain est à toi. Tu gardes la main et tu choisis ensuite à qui donner, de façon encadrée.</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Engagement juridique, régime matrimonial à choisir.</t>
+          <t>Ta copine n'est pas héritière sans mariage ni testament. Des dons à une personne non mariée ou non pacsée sont taxés lourdement.</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Contrat de mariage, testament</t>
+          <t>Droits de donation / succession entre non-mariés</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
+          <t>Aux deux noms (copine)</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Le gain est partagé dès le départ.</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Co-propriété : en cas de séparation, c'est compliqué. Aussi une donation indirecte possible. Ça ne règle pas la transmission.</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Notaire AVANT de signer</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>À ton nom + PACS ou mariage</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Le conjoint ou partenaire pacsé est exonéré de droits de succession. Le mariage protège davantage.</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Engagement juridique, régime matrimonial à choisir.</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Contrat de mariage, testament</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
           <t>À ton nom + assurance-vie</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>Tu désignes qui reçoit, hors succession classique, avec un abattement par bénéficiaire (152 500 € dans le cas général, à vérifier).</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>Clause bénéficiaire à rédiger précisément. Fiscalité selon l'âge des versements.</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>Clause bénéficiaire avec le notaire</t>
         </is>
@@ -3851,7 +3888,7 @@
     <mergeCell ref="A1:D1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="D4:D14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D4:D16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Oui,Non"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>